<commit_message>
Update UPVC- END PLUG to UPVC CIRCUIT PLUG and remove sizes/packing
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -17220,10 +17220,10 @@
         <v>-</v>
       </c>
       <c r="C481" t="str">
-        <v>UPVC- END PLUG (1/2)</v>
+        <v>UPVC CIRCUIT PLUG</v>
       </c>
       <c r="D481" t="str">
-        <v>UPVC- END PLUG</v>
+        <v>UPVC CIRCUIT PLUG</v>
       </c>
       <c r="E481" t="str">
         <v>UPVC Pipes &amp; Fittings</v>
@@ -17232,7 +17232,7 @@
         <v>General</v>
       </c>
       <c r="G481" t="str">
-        <v>1/2</v>
+        <v>Standard</v>
       </c>
       <c r="H481" t="str">
         <v>BOX</v>
@@ -17244,7 +17244,7 @@
         <v>Active</v>
       </c>
       <c r="K481" t="str">
-        <v>UPVC- END PLUG. Available sizes: 1/2.</v>
+        <v>UPVC CIRCUIT PLUG.</v>
       </c>
     </row>
     <row r="482">

</xml_diff>

<commit_message>
Update UPVC CIRCUIT PLUG variant (1/2: FG-400402, Packing: 300)
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -17217,10 +17217,10 @@
         <v>480</v>
       </c>
       <c r="B481" t="str">
-        <v>-</v>
+        <v>FG-400402</v>
       </c>
       <c r="C481" t="str">
-        <v>UPVC CIRCUIT PLUG</v>
+        <v>UPVC CIRCUIT PLUG (1/2)</v>
       </c>
       <c r="D481" t="str">
         <v>UPVC CIRCUIT PLUG</v>
@@ -17232,19 +17232,19 @@
         <v>General</v>
       </c>
       <c r="G481" t="str">
-        <v>Standard</v>
+        <v>1/2</v>
       </c>
       <c r="H481" t="str">
         <v>BOX</v>
       </c>
-      <c r="I481" t="str">
-        <v>-</v>
+      <c r="I481">
+        <v>300</v>
       </c>
       <c r="J481" t="str">
         <v>Active</v>
       </c>
       <c r="K481" t="str">
-        <v>UPVC CIRCUIT PLUG.</v>
+        <v>UPVC CIRCUIT PLUG. Available sizes: 1/2.</v>
       </c>
     </row>
     <row r="482">

</xml_diff>

<commit_message>
Update PN10 - REDUCING BUSH ISI to AGRI REDUCING BUSH 10KG with variants and product codes
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -36152,13 +36152,13 @@
         <v>1021</v>
       </c>
       <c r="B1022" t="str">
-        <v>-</v>
+        <v>FG-400673</v>
       </c>
       <c r="C1022" t="str">
-        <v>PN10 - REDUCING BUSH ISI (32 X 20)</v>
+        <v>AGRI REDUCING BUSH 10KG (32 X 20MM)</v>
       </c>
       <c r="D1022" t="str">
-        <v>PN10 - REDUCING BUSH ISI</v>
+        <v>AGRI REDUCING BUSH 10KG</v>
       </c>
       <c r="E1022" t="str">
         <v>Agriculture Pipes &amp; Fittings</v>
@@ -36167,19 +36167,19 @@
         <v>General</v>
       </c>
       <c r="G1022" t="str">
-        <v>32 X 20</v>
+        <v>32 X 20MM</v>
       </c>
       <c r="H1022" t="str">
         <v>BOX</v>
       </c>
-      <c r="I1022" t="str">
-        <v>-</v>
+      <c r="I1022">
+        <v>250</v>
       </c>
       <c r="J1022" t="str">
         <v>Active</v>
       </c>
       <c r="K1022" t="str">
-        <v>PN10 - REDUCING BUSH ISI for agriculture irrigation and piping systems.</v>
+        <v>AGRI REDUCING BUSH 10KG. Available sizes: 32 X 20MM, 32 X 25MM.</v>
       </c>
     </row>
     <row r="1023">
@@ -36187,13 +36187,13 @@
         <v>1022</v>
       </c>
       <c r="B1023" t="str">
-        <v>-</v>
+        <v>FG-400674</v>
       </c>
       <c r="C1023" t="str">
-        <v>PN10 - REDUCING BUSH ISI (32 X 25)</v>
+        <v>AGRI REDUCING BUSH 10KG (32 X 25MM)</v>
       </c>
       <c r="D1023" t="str">
-        <v>PN10 - REDUCING BUSH ISI</v>
+        <v>AGRI REDUCING BUSH 10KG</v>
       </c>
       <c r="E1023" t="str">
         <v>Agriculture Pipes &amp; Fittings</v>
@@ -36202,19 +36202,19 @@
         <v>General</v>
       </c>
       <c r="G1023" t="str">
-        <v>32 X 25</v>
+        <v>32 X 25MM</v>
       </c>
       <c r="H1023" t="str">
         <v>BOX</v>
       </c>
-      <c r="I1023" t="str">
-        <v>-</v>
+      <c r="I1023">
+        <v>250</v>
       </c>
       <c r="J1023" t="str">
         <v>Active</v>
       </c>
       <c r="K1023" t="str">
-        <v>PN10 - REDUCING BUSH ISI for agriculture irrigation and piping systems.</v>
+        <v>AGRI REDUCING BUSH 10KG. Available sizes: 32 X 20MM, 32 X 25MM.</v>
       </c>
     </row>
     <row r="1024">

</xml_diff>

<commit_message>
Update 3M STANDARD PLUS PIPE to COLOUMN PIPE COUPLER STANDARD PLUS and remove sizes/packing
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -43085,10 +43085,10 @@
         <v>-</v>
       </c>
       <c r="C1220" t="str">
-        <v>3M STANDARD PLUS PIPE (60MM 25 COUPLER TYPE)</v>
+        <v>COLOUMN PIPE COUPLER STANDARD PLUS</v>
       </c>
       <c r="D1220" t="str">
-        <v>3M STANDARD PLUS PIPE</v>
+        <v>COLOUMN PIPE COUPLER STANDARD PLUS</v>
       </c>
       <c r="E1220" t="str">
         <v>UPVC COLUMN PIPES</v>
@@ -43097,7 +43097,7 @@
         <v>General</v>
       </c>
       <c r="G1220" t="str">
-        <v>60MM 25 COUPLER TYPE</v>
+        <v>Standard</v>
       </c>
       <c r="H1220" t="str">
         <v>MTR</v>
@@ -43109,7 +43109,7 @@
         <v>Active</v>
       </c>
       <c r="K1220" t="str">
-        <v>3M Standard Plus UPVC Column Pipe for submersible pump systems.</v>
+        <v>COLOUMN PIPE COUPLER STANDARD PLUS.</v>
       </c>
     </row>
     <row r="1221">

</xml_diff>

<commit_message>
Update COLOUMN PIPE COUPLER STANDARD PLUS variant (2 25KG: FG-401173) and packing data
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -43082,10 +43082,10 @@
         <v>1219</v>
       </c>
       <c r="B1220" t="str">
-        <v>-</v>
+        <v>FG-401173</v>
       </c>
       <c r="C1220" t="str">
-        <v>COLOUMN PIPE COUPLER STANDARD PLUS</v>
+        <v>COLOUMN PIPE COUPLER STANDARD PLUS (2 25KG)</v>
       </c>
       <c r="D1220" t="str">
         <v>COLOUMN PIPE COUPLER STANDARD PLUS</v>
@@ -43097,19 +43097,19 @@
         <v>General</v>
       </c>
       <c r="G1220" t="str">
-        <v>Standard</v>
+        <v>2 25KG</v>
       </c>
       <c r="H1220" t="str">
         <v>MTR</v>
       </c>
-      <c r="I1220" t="str">
-        <v>-</v>
+      <c r="I1220">
+        <v>12</v>
       </c>
       <c r="J1220" t="str">
         <v>Active</v>
       </c>
       <c r="K1220" t="str">
-        <v>COLOUMN PIPE COUPLER STANDARD PLUS.</v>
+        <v>COLOUMN PIPE COUPLER STANDARD PLUS. Available sizes: 2 25KG.</v>
       </c>
     </row>
     <row r="1221">

</xml_diff>

<commit_message>
Update COLOUMN PIPE COUPLER STANDARD PLUS to COLOUMN PIPE STANDARD PLUS and remove sizes/packing
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -43082,13 +43082,13 @@
         <v>1219</v>
       </c>
       <c r="B1220" t="str">
-        <v>FG-401173</v>
+        <v>-</v>
       </c>
       <c r="C1220" t="str">
-        <v>COLOUMN PIPE COUPLER STANDARD PLUS (2 25KG)</v>
+        <v>COLOUMN PIPE STANDARD PLUS</v>
       </c>
       <c r="D1220" t="str">
-        <v>COLOUMN PIPE COUPLER STANDARD PLUS</v>
+        <v>COLOUMN PIPE STANDARD PLUS</v>
       </c>
       <c r="E1220" t="str">
         <v>UPVC COLUMN PIPES</v>
@@ -43097,19 +43097,19 @@
         <v>General</v>
       </c>
       <c r="G1220" t="str">
-        <v>2 25KG</v>
+        <v>Standard</v>
       </c>
       <c r="H1220" t="str">
         <v>MTR</v>
       </c>
-      <c r="I1220">
-        <v>12</v>
+      <c r="I1220" t="str">
+        <v>-</v>
       </c>
       <c r="J1220" t="str">
         <v>Active</v>
       </c>
       <c r="K1220" t="str">
-        <v>COLOUMN PIPE COUPLER STANDARD PLUS. Available sizes: 2 25KG.</v>
+        <v>COLOUMN PIPE STANDARD PLUS.</v>
       </c>
     </row>
     <row r="1221">

</xml_diff>

<commit_message>
Update COLOUMN PIPE STANDARD PLUS variant (60MM 2 Inch 25KG COUPLER TYPE: FG-401173, Packing 12)
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -43082,10 +43082,10 @@
         <v>1219</v>
       </c>
       <c r="B1220" t="str">
-        <v>-</v>
+        <v>FG-401173</v>
       </c>
       <c r="C1220" t="str">
-        <v>COLOUMN PIPE STANDARD PLUS</v>
+        <v>COLOUMN PIPE STANDARD PLUS (60MM 2 Inch 25KG COUPLER TYPE)</v>
       </c>
       <c r="D1220" t="str">
         <v>COLOUMN PIPE STANDARD PLUS</v>
@@ -43097,19 +43097,19 @@
         <v>General</v>
       </c>
       <c r="G1220" t="str">
-        <v>Standard</v>
+        <v>60MM 2 Inch 25KG COUPLER TYPE</v>
       </c>
       <c r="H1220" t="str">
         <v>MTR</v>
       </c>
-      <c r="I1220" t="str">
-        <v>-</v>
+      <c r="I1220">
+        <v>12</v>
       </c>
       <c r="J1220" t="str">
         <v>Active</v>
       </c>
       <c r="K1220" t="str">
-        <v>COLOUMN PIPE STANDARD PLUS.</v>
+        <v>COLOUMN PIPE STANDARD PLUS. Available sizes: 60MM 2 Inch 25KG COUPLER TYPE.</v>
       </c>
     </row>
     <row r="1221">

</xml_diff>

<commit_message>
Add DWC PIPE SN4 and DWC PIPE SN8 products under DWC category
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1340"/>
+  <dimension ref="A1:K1342"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -47312,9 +47312,79 @@
         <v>EWC Toilet Seat Cover without jet spray.</v>
       </c>
     </row>
+    <row r="1341">
+      <c r="A1341">
+        <v>1340</v>
+      </c>
+      <c r="B1341" t="str">
+        <v>-</v>
+      </c>
+      <c r="C1341" t="str">
+        <v>DWC PIPE SN4</v>
+      </c>
+      <c r="D1341" t="str">
+        <v>DWC PIPE SN4</v>
+      </c>
+      <c r="E1341" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1341" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1341" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="H1341" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1341" t="str">
+        <v>-</v>
+      </c>
+      <c r="J1341" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1341" t="str">
+        <v>DWC PIPE SN4 for underground cable protection and drainage systems.</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342">
+        <v>1341</v>
+      </c>
+      <c r="B1342" t="str">
+        <v>-</v>
+      </c>
+      <c r="C1342" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="D1342" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="E1342" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1342" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1342" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="H1342" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1342" t="str">
+        <v>-</v>
+      </c>
+      <c r="J1342" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1342" t="str">
+        <v>DWC PIPE SN8 for underground cable protection and drainage systems.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K1340"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K1342"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update DWC PIPE SN4 variants (150MM-500MM) with product codes
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1342"/>
+  <dimension ref="A1:K1347"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -47317,10 +47317,10 @@
         <v>1340</v>
       </c>
       <c r="B1341" t="str">
-        <v>-</v>
+        <v>FG-401854</v>
       </c>
       <c r="C1341" t="str">
-        <v>DWC PIPE SN4</v>
+        <v>DWC PIPE SN4 (150MM)</v>
       </c>
       <c r="D1341" t="str">
         <v>DWC PIPE SN4</v>
@@ -47332,19 +47332,19 @@
         <v>General</v>
       </c>
       <c r="G1341" t="str">
-        <v>Standard</v>
+        <v>150MM</v>
       </c>
       <c r="H1341" t="str">
         <v>MTR</v>
       </c>
-      <c r="I1341" t="str">
-        <v>-</v>
+      <c r="I1341">
+        <v>1</v>
       </c>
       <c r="J1341" t="str">
         <v>Active</v>
       </c>
       <c r="K1341" t="str">
-        <v>DWC PIPE SN4 for underground cable protection and drainage systems.</v>
+        <v>DWC PIPE SN4 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
       </c>
     </row>
     <row r="1342">
@@ -47352,13 +47352,13 @@
         <v>1341</v>
       </c>
       <c r="B1342" t="str">
-        <v>-</v>
+        <v>FG-401855</v>
       </c>
       <c r="C1342" t="str">
-        <v>DWC PIPE SN8</v>
+        <v>DWC PIPE SN4 (200MM)</v>
       </c>
       <c r="D1342" t="str">
-        <v>DWC PIPE SN8</v>
+        <v>DWC PIPE SN4</v>
       </c>
       <c r="E1342" t="str">
         <v>DWC</v>
@@ -47367,24 +47367,199 @@
         <v>General</v>
       </c>
       <c r="G1342" t="str">
-        <v>Standard</v>
+        <v>200MM</v>
       </c>
       <c r="H1342" t="str">
         <v>MTR</v>
       </c>
-      <c r="I1342" t="str">
-        <v>-</v>
+      <c r="I1342">
+        <v>1</v>
       </c>
       <c r="J1342" t="str">
         <v>Active</v>
       </c>
       <c r="K1342" t="str">
+        <v>DWC PIPE SN4 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343">
+        <v>1342</v>
+      </c>
+      <c r="B1343" t="str">
+        <v>FG-401856</v>
+      </c>
+      <c r="C1343" t="str">
+        <v>DWC PIPE SN4 (250MM)</v>
+      </c>
+      <c r="D1343" t="str">
+        <v>DWC PIPE SN4</v>
+      </c>
+      <c r="E1343" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1343" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1343" t="str">
+        <v>250MM</v>
+      </c>
+      <c r="H1343" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1343">
+        <v>1</v>
+      </c>
+      <c r="J1343" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1343" t="str">
+        <v>DWC PIPE SN4 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344">
+        <v>1343</v>
+      </c>
+      <c r="B1344" t="str">
+        <v>FG-401857</v>
+      </c>
+      <c r="C1344" t="str">
+        <v>DWC PIPE SN4 (300MM)</v>
+      </c>
+      <c r="D1344" t="str">
+        <v>DWC PIPE SN4</v>
+      </c>
+      <c r="E1344" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1344" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1344" t="str">
+        <v>300MM</v>
+      </c>
+      <c r="H1344" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1344">
+        <v>1</v>
+      </c>
+      <c r="J1344" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1344" t="str">
+        <v>DWC PIPE SN4 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345">
+        <v>1344</v>
+      </c>
+      <c r="B1345" t="str">
+        <v>FG-401858</v>
+      </c>
+      <c r="C1345" t="str">
+        <v>DWC PIPE SN4 (400MM)</v>
+      </c>
+      <c r="D1345" t="str">
+        <v>DWC PIPE SN4</v>
+      </c>
+      <c r="E1345" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1345" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1345" t="str">
+        <v>400MM</v>
+      </c>
+      <c r="H1345" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1345">
+        <v>1</v>
+      </c>
+      <c r="J1345" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1345" t="str">
+        <v>DWC PIPE SN4 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346">
+        <v>1345</v>
+      </c>
+      <c r="B1346" t="str">
+        <v>FG-401859</v>
+      </c>
+      <c r="C1346" t="str">
+        <v>DWC PIPE SN4 (500MM)</v>
+      </c>
+      <c r="D1346" t="str">
+        <v>DWC PIPE SN4</v>
+      </c>
+      <c r="E1346" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1346" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1346" t="str">
+        <v>500MM</v>
+      </c>
+      <c r="H1346" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1346">
+        <v>1</v>
+      </c>
+      <c r="J1346" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1346" t="str">
+        <v>DWC PIPE SN4 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347">
+        <v>1346</v>
+      </c>
+      <c r="B1347" t="str">
+        <v>-</v>
+      </c>
+      <c r="C1347" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="D1347" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="E1347" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1347" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1347" t="str">
+        <v>Standard</v>
+      </c>
+      <c r="H1347" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1347" t="str">
+        <v>-</v>
+      </c>
+      <c r="J1347" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1347" t="str">
         <v>DWC PIPE SN8 for underground cable protection and drainage systems.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K1342"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K1347"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update DWC PIPE SN8 variants (150MM-500MM) with product codes
</commit_message>
<xml_diff>
--- a/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
+++ b/public/Gouri_Aqua_Plast_Products_Catalog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1347"/>
+  <dimension ref="A1:K1352"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -47527,10 +47527,10 @@
         <v>1346</v>
       </c>
       <c r="B1347" t="str">
-        <v>-</v>
+        <v>FG-401860</v>
       </c>
       <c r="C1347" t="str">
-        <v>DWC PIPE SN8</v>
+        <v>DWC PIPE SN8 (150MM)</v>
       </c>
       <c r="D1347" t="str">
         <v>DWC PIPE SN8</v>
@@ -47542,24 +47542,199 @@
         <v>General</v>
       </c>
       <c r="G1347" t="str">
-        <v>Standard</v>
+        <v>150MM</v>
       </c>
       <c r="H1347" t="str">
         <v>MTR</v>
       </c>
-      <c r="I1347" t="str">
-        <v>-</v>
+      <c r="I1347">
+        <v>1</v>
       </c>
       <c r="J1347" t="str">
         <v>Active</v>
       </c>
       <c r="K1347" t="str">
-        <v>DWC PIPE SN8 for underground cable protection and drainage systems.</v>
+        <v>DWC PIPE SN8 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348">
+        <v>1347</v>
+      </c>
+      <c r="B1348" t="str">
+        <v>FG-401861</v>
+      </c>
+      <c r="C1348" t="str">
+        <v>DWC PIPE SN8 (200MM)</v>
+      </c>
+      <c r="D1348" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="E1348" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1348" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1348" t="str">
+        <v>200MM</v>
+      </c>
+      <c r="H1348" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1348">
+        <v>1</v>
+      </c>
+      <c r="J1348" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1348" t="str">
+        <v>DWC PIPE SN8 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349">
+        <v>1348</v>
+      </c>
+      <c r="B1349" t="str">
+        <v>FG-401862</v>
+      </c>
+      <c r="C1349" t="str">
+        <v>DWC PIPE SN8 (250MM)</v>
+      </c>
+      <c r="D1349" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="E1349" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1349" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1349" t="str">
+        <v>250MM</v>
+      </c>
+      <c r="H1349" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1349">
+        <v>1</v>
+      </c>
+      <c r="J1349" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1349" t="str">
+        <v>DWC PIPE SN8 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350">
+        <v>1349</v>
+      </c>
+      <c r="B1350" t="str">
+        <v>FG-401863</v>
+      </c>
+      <c r="C1350" t="str">
+        <v>DWC PIPE SN8 (300MM)</v>
+      </c>
+      <c r="D1350" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="E1350" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1350" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1350" t="str">
+        <v>300MM</v>
+      </c>
+      <c r="H1350" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1350">
+        <v>1</v>
+      </c>
+      <c r="J1350" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1350" t="str">
+        <v>DWC PIPE SN8 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351">
+        <v>1350</v>
+      </c>
+      <c r="B1351" t="str">
+        <v>FG-401864</v>
+      </c>
+      <c r="C1351" t="str">
+        <v>DWC PIPE SN8 (400MM)</v>
+      </c>
+      <c r="D1351" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="E1351" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1351" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1351" t="str">
+        <v>400MM</v>
+      </c>
+      <c r="H1351" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1351">
+        <v>1</v>
+      </c>
+      <c r="J1351" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1351" t="str">
+        <v>DWC PIPE SN8 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352">
+        <v>1351</v>
+      </c>
+      <c r="B1352" t="str">
+        <v>FG-401865</v>
+      </c>
+      <c r="C1352" t="str">
+        <v>DWC PIPE SN8 (500MM)</v>
+      </c>
+      <c r="D1352" t="str">
+        <v>DWC PIPE SN8</v>
+      </c>
+      <c r="E1352" t="str">
+        <v>DWC</v>
+      </c>
+      <c r="F1352" t="str">
+        <v>General</v>
+      </c>
+      <c r="G1352" t="str">
+        <v>500MM</v>
+      </c>
+      <c r="H1352" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="I1352">
+        <v>1</v>
+      </c>
+      <c r="J1352" t="str">
+        <v>Active</v>
+      </c>
+      <c r="K1352" t="str">
+        <v>DWC PIPE SN8 for underground cable protection and drainage systems. Available sizes: 150MM, 200MM, 250MM, 300MM, 400MM, 500MM.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K1347"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K1352"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>